<commit_message>
Add exception management fields and root cause tracking
</commit_message>
<xml_diff>
--- a/output/Investment_Operations_Exception_Report.xlsx
+++ b/output/Investment_Operations_Exception_Report.xlsx
@@ -15,6 +15,7 @@
     <sheet name="High Risk Exceptions" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Portfolio Breakdown" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="Source Breakdown" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Root Cause Breakdown" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -420,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -513,6 +514,26 @@
       </c>
       <c r="B9" t="n">
         <v>486554</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Critical Priority Exceptions</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Average Days Open</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>2.5</v>
       </c>
     </row>
   </sheetData>
@@ -526,7 +547,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L16"/>
+  <dimension ref="A1:P16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -582,10 +603,30 @@
       </c>
       <c r="K1" t="inlineStr">
         <is>
+          <t>priority</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>exception_owner</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>days_open</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>root_cause_category</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
           <t>recommended_action</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
@@ -638,10 +679,28 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Trade Operations Team</t>
+        </is>
+      </c>
+      <c r="M2" t="n">
+        <v>2</v>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>Allocation Issue</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
           <t>Compare internal allocation records against custodian position or trade details.</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="P2" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -698,10 +757,28 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Trade Operations Team</t>
+        </is>
+      </c>
+      <c r="M3" t="n">
+        <v>3</v>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Settlement Issue</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
           <t>Confirm contractual settlement date and update the incorrect record.</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="P3" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -758,10 +835,28 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Trade Operations Team</t>
+        </is>
+      </c>
+      <c r="M4" t="n">
+        <v>2</v>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Booking Issue</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
           <t>Confirm record with custodian and investigate whether the position or trade failed to book externally.</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="P4" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -814,10 +909,28 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Trade Operations Team</t>
+        </is>
+      </c>
+      <c r="M5" t="n">
+        <v>2</v>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>Pricing Issue</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
           <t>Review execution price, broker confirmation, and custodian booking details.</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr">
+      <c r="P5" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -874,10 +987,28 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Trade Operations Team</t>
+        </is>
+      </c>
+      <c r="M6" t="n">
+        <v>2</v>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>Booking Issue</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
           <t>Confirm record with custodian and investigate whether the position or trade failed to book externally.</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr">
+      <c r="P6" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -934,10 +1065,28 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>Trade Operations Team</t>
+        </is>
+      </c>
+      <c r="M7" t="n">
+        <v>2</v>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>Booking Issue</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
           <t>Confirm record with custodian and investigate whether the position or trade failed to book externally.</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr">
+      <c r="P7" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -994,10 +1143,28 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>Trade Operations Team</t>
+        </is>
+      </c>
+      <c r="M8" t="n">
+        <v>2</v>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>Booking Issue</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
           <t>Review custodian activity and confirm whether the record should be booked internally.</t>
         </is>
       </c>
-      <c r="L8" t="inlineStr">
+      <c r="P8" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -1050,10 +1217,28 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>Portfolio Accounting Team</t>
+        </is>
+      </c>
+      <c r="M9" t="n">
+        <v>3</v>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>Pricing Issue</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
           <t>Review pricing source, valuation date, and custodian market price feed.</t>
         </is>
       </c>
-      <c r="L9" t="inlineStr">
+      <c r="P9" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -1110,10 +1295,28 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>Portfolio Accounting Team</t>
+        </is>
+      </c>
+      <c r="M10" t="n">
+        <v>2</v>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>Booking Issue</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
           <t>Review custodian activity and confirm whether the record should be booked internally.</t>
         </is>
       </c>
-      <c r="L10" t="inlineStr">
+      <c r="P10" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -1170,10 +1373,28 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>Portfolio Accounting Team</t>
+        </is>
+      </c>
+      <c r="M11" t="n">
+        <v>2</v>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>Booking Issue</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
           <t>Confirm record with custodian and investigate whether the position or trade failed to book externally.</t>
         </is>
       </c>
-      <c r="L11" t="inlineStr">
+      <c r="P11" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -1226,10 +1447,28 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>Portfolio Accounting Team</t>
+        </is>
+      </c>
+      <c r="M12" t="n">
+        <v>4</v>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>Allocation Issue</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
           <t>Compare internal allocation records against custodian position or trade details.</t>
         </is>
       </c>
-      <c r="L12" t="inlineStr">
+      <c r="P12" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -1286,10 +1525,28 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>Portfolio Accounting Team</t>
+        </is>
+      </c>
+      <c r="M13" t="n">
+        <v>4</v>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>Booking Issue</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
           <t>Confirm record with custodian and investigate whether the position or trade failed to book externally.</t>
         </is>
       </c>
-      <c r="L13" t="inlineStr">
+      <c r="P13" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -1342,10 +1599,28 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>Portfolio Accounting Team</t>
+        </is>
+      </c>
+      <c r="M14" t="n">
+        <v>4</v>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>Allocation Issue</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
           <t>Compare internal allocation records against custodian position or trade details.</t>
         </is>
       </c>
-      <c r="L14" t="inlineStr">
+      <c r="P14" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -1398,10 +1673,28 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>Cash Operations Team</t>
+        </is>
+      </c>
+      <c r="M15" t="n">
+        <v>2</v>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>Cash Movement Issue</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
           <t>Investigate unsettled trades, custodian cash movements, fees, and income activity causing the cash difference.</t>
         </is>
       </c>
-      <c r="L15" t="inlineStr">
+      <c r="P15" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -1454,10 +1747,28 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>Cash Operations Team</t>
+        </is>
+      </c>
+      <c r="M16" t="n">
+        <v>2</v>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>Cash Movement Issue</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
           <t>Investigate unsettled trades, custodian cash movements, fees, and income activity causing the cash difference.</t>
         </is>
       </c>
-      <c r="L16" t="inlineStr">
+      <c r="P16" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -1474,7 +1785,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:P8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1530,10 +1841,30 @@
       </c>
       <c r="K1" t="inlineStr">
         <is>
+          <t>priority</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>exception_owner</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>days_open</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>root_cause_category</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
           <t>recommended_action</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
@@ -1586,10 +1917,28 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Trade Operations Team</t>
+        </is>
+      </c>
+      <c r="M2" t="n">
+        <v>2</v>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>Allocation Issue</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
           <t>Compare internal allocation records against custodian position or trade details.</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="P2" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -1646,10 +1995,28 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Trade Operations Team</t>
+        </is>
+      </c>
+      <c r="M3" t="n">
+        <v>3</v>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Settlement Issue</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
           <t>Confirm contractual settlement date and update the incorrect record.</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="P3" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -1706,10 +2073,28 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Trade Operations Team</t>
+        </is>
+      </c>
+      <c r="M4" t="n">
+        <v>2</v>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Booking Issue</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
           <t>Confirm record with custodian and investigate whether the position or trade failed to book externally.</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="P4" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -1762,10 +2147,28 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Trade Operations Team</t>
+        </is>
+      </c>
+      <c r="M5" t="n">
+        <v>2</v>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>Pricing Issue</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
           <t>Review execution price, broker confirmation, and custodian booking details.</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr">
+      <c r="P5" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -1822,10 +2225,28 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Trade Operations Team</t>
+        </is>
+      </c>
+      <c r="M6" t="n">
+        <v>2</v>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>Booking Issue</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
           <t>Confirm record with custodian and investigate whether the position or trade failed to book externally.</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr">
+      <c r="P6" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -1882,10 +2303,28 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>Trade Operations Team</t>
+        </is>
+      </c>
+      <c r="M7" t="n">
+        <v>2</v>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>Booking Issue</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
           <t>Confirm record with custodian and investigate whether the position or trade failed to book externally.</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr">
+      <c r="P7" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -1942,10 +2381,28 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>Trade Operations Team</t>
+        </is>
+      </c>
+      <c r="M8" t="n">
+        <v>2</v>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>Booking Issue</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
           <t>Review custodian activity and confirm whether the record should be booked internally.</t>
         </is>
       </c>
-      <c r="L8" t="inlineStr">
+      <c r="P8" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -1962,7 +2419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:P7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2018,10 +2475,30 @@
       </c>
       <c r="K1" t="inlineStr">
         <is>
+          <t>priority</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>exception_owner</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>days_open</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>root_cause_category</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
           <t>recommended_action</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
@@ -2074,10 +2551,28 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Portfolio Accounting Team</t>
+        </is>
+      </c>
+      <c r="M2" t="n">
+        <v>3</v>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>Pricing Issue</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
           <t>Review pricing source, valuation date, and custodian market price feed.</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="P2" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -2134,10 +2629,28 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Portfolio Accounting Team</t>
+        </is>
+      </c>
+      <c r="M3" t="n">
+        <v>2</v>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Booking Issue</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
           <t>Review custodian activity and confirm whether the record should be booked internally.</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="P3" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -2194,10 +2707,28 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Portfolio Accounting Team</t>
+        </is>
+      </c>
+      <c r="M4" t="n">
+        <v>2</v>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Booking Issue</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
           <t>Confirm record with custodian and investigate whether the position or trade failed to book externally.</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="P4" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -2250,10 +2781,28 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Portfolio Accounting Team</t>
+        </is>
+      </c>
+      <c r="M5" t="n">
+        <v>4</v>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>Allocation Issue</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
           <t>Compare internal allocation records against custodian position or trade details.</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr">
+      <c r="P5" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -2310,10 +2859,28 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Portfolio Accounting Team</t>
+        </is>
+      </c>
+      <c r="M6" t="n">
+        <v>4</v>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>Booking Issue</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
           <t>Confirm record with custodian and investigate whether the position or trade failed to book externally.</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr">
+      <c r="P6" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -2366,10 +2933,28 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>Portfolio Accounting Team</t>
+        </is>
+      </c>
+      <c r="M7" t="n">
+        <v>4</v>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>Allocation Issue</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
           <t>Compare internal allocation records against custodian position or trade details.</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr">
+      <c r="P7" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -2386,7 +2971,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:P3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2442,10 +3027,30 @@
       </c>
       <c r="K1" t="inlineStr">
         <is>
+          <t>priority</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>exception_owner</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>days_open</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>root_cause_category</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
           <t>recommended_action</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
@@ -2498,10 +3103,28 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Cash Operations Team</t>
+        </is>
+      </c>
+      <c r="M2" t="n">
+        <v>2</v>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>Cash Movement Issue</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
           <t>Investigate unsettled trades, custodian cash movements, fees, and income activity causing the cash difference.</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="P2" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -2554,10 +3177,28 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Cash Operations Team</t>
+        </is>
+      </c>
+      <c r="M3" t="n">
+        <v>2</v>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Cash Movement Issue</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
           <t>Investigate unsettled trades, custodian cash movements, fees, and income activity causing the cash difference.</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="P3" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -2574,7 +3215,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L14"/>
+  <dimension ref="A1:P14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2630,10 +3271,30 @@
       </c>
       <c r="K1" t="inlineStr">
         <is>
+          <t>priority</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>exception_owner</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>days_open</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>root_cause_category</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
           <t>recommended_action</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
@@ -2686,10 +3347,28 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Portfolio Accounting Team</t>
+        </is>
+      </c>
+      <c r="M2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>Allocation Issue</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
           <t>Compare internal allocation records against custodian position or trade details.</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="P2" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -2746,10 +3425,28 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Portfolio Accounting Team</t>
+        </is>
+      </c>
+      <c r="M3" t="n">
+        <v>4</v>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Booking Issue</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
           <t>Confirm record with custodian and investigate whether the position or trade failed to book externally.</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="P3" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -2802,10 +3499,28 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Portfolio Accounting Team</t>
+        </is>
+      </c>
+      <c r="M4" t="n">
+        <v>4</v>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Allocation Issue</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
           <t>Compare internal allocation records against custodian position or trade details.</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="P4" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -2858,10 +3573,28 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Trade Operations Team</t>
+        </is>
+      </c>
+      <c r="M5" t="n">
+        <v>2</v>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>Allocation Issue</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
           <t>Compare internal allocation records against custodian position or trade details.</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr">
+      <c r="P5" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -2918,10 +3651,28 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Trade Operations Team</t>
+        </is>
+      </c>
+      <c r="M6" t="n">
+        <v>2</v>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>Booking Issue</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
           <t>Confirm record with custodian and investigate whether the position or trade failed to book externally.</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr">
+      <c r="P6" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -2974,10 +3725,28 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>Cash Operations Team</t>
+        </is>
+      </c>
+      <c r="M7" t="n">
+        <v>2</v>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>Cash Movement Issue</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
           <t>Investigate unsettled trades, custodian cash movements, fees, and income activity causing the cash difference.</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr">
+      <c r="P7" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -3034,10 +3803,28 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>Portfolio Accounting Team</t>
+        </is>
+      </c>
+      <c r="M8" t="n">
+        <v>2</v>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>Booking Issue</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
           <t>Confirm record with custodian and investigate whether the position or trade failed to book externally.</t>
         </is>
       </c>
-      <c r="L8" t="inlineStr">
+      <c r="P8" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -3090,10 +3877,28 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>Trade Operations Team</t>
+        </is>
+      </c>
+      <c r="M9" t="n">
+        <v>2</v>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>Pricing Issue</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
           <t>Review execution price, broker confirmation, and custodian booking details.</t>
         </is>
       </c>
-      <c r="L9" t="inlineStr">
+      <c r="P9" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -3150,10 +3955,28 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>Portfolio Accounting Team</t>
+        </is>
+      </c>
+      <c r="M10" t="n">
+        <v>2</v>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>Booking Issue</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
           <t>Review custodian activity and confirm whether the record should be booked internally.</t>
         </is>
       </c>
-      <c r="L10" t="inlineStr">
+      <c r="P10" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -3210,10 +4033,28 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>Trade Operations Team</t>
+        </is>
+      </c>
+      <c r="M11" t="n">
+        <v>2</v>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>Booking Issue</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
           <t>Review custodian activity and confirm whether the record should be booked internally.</t>
         </is>
       </c>
-      <c r="L11" t="inlineStr">
+      <c r="P11" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -3266,10 +4107,28 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>Cash Operations Team</t>
+        </is>
+      </c>
+      <c r="M12" t="n">
+        <v>2</v>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>Cash Movement Issue</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
           <t>Investigate unsettled trades, custodian cash movements, fees, and income activity causing the cash difference.</t>
         </is>
       </c>
-      <c r="L12" t="inlineStr">
+      <c r="P12" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -3326,10 +4185,28 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>Trade Operations Team</t>
+        </is>
+      </c>
+      <c r="M13" t="n">
+        <v>2</v>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>Booking Issue</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
           <t>Confirm record with custodian and investigate whether the position or trade failed to book externally.</t>
         </is>
       </c>
-      <c r="L13" t="inlineStr">
+      <c r="P13" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -3386,10 +4263,28 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>Trade Operations Team</t>
+        </is>
+      </c>
+      <c r="M14" t="n">
+        <v>2</v>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>Booking Issue</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
           <t>Confirm record with custodian and investigate whether the position or trade failed to book externally.</t>
         </is>
       </c>
-      <c r="L14" t="inlineStr">
+      <c r="P14" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -3552,4 +4447,100 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>root_cause_category</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>exception_count</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>estimated_dollar_impact</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Allocation Issue</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C2" t="n">
+        <v>214417.5</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Booking Issue</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>7</v>
+      </c>
+      <c r="C3" t="n">
+        <v>155435</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Pricing Issue</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C4" t="n">
+        <v>63596.5</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Cash Movement Issue</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>2</v>
+      </c>
+      <c r="C5" t="n">
+        <v>34845</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Settlement Issue</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C6" t="n">
+        <v>18260</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Connect expanded holdings dataset to reconciliation engine
</commit_message>
<xml_diff>
--- a/output/Investment_Operations_Exception_Report.xlsx
+++ b/output/Investment_Operations_Exception_Report.xlsx
@@ -443,7 +443,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="3">
@@ -453,7 +453,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4">
@@ -483,7 +483,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="7">
@@ -493,7 +493,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="8">
@@ -513,7 +513,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>486554</v>
+        <v>729893.5</v>
       </c>
     </row>
     <row r="10">
@@ -533,7 +533,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>2.5</v>
+        <v>2.6</v>
       </c>
     </row>
   </sheetData>
@@ -547,7 +547,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P16"/>
+  <dimension ref="A1:P18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -640,17 +640,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>T002</t>
+          <t>T0007</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Growth Fund</t>
+          <t>Short Duration Bond Fund</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>JPM</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -664,13 +664,13 @@
         </is>
       </c>
       <c r="G2" t="n">
-        <v>75</v>
+        <v>200</v>
       </c>
       <c r="H2" t="n">
-        <v>70</v>
+        <v>175</v>
       </c>
       <c r="I2" t="n">
-        <v>31507.5</v>
+        <v>41094</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -714,50 +714,46 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>T004</t>
+          <t>T0012</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Income Fund</t>
+          <t>Core Income Fund</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>TLT</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Bond ETF</t>
+          <t>Equity</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>settlement_date_mismatch</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>2026-06-04</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>2026-06-05</t>
-        </is>
+          <t>price_mismatch</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>417.69</v>
+      </c>
+      <c r="H3" t="n">
+        <v>418.04</v>
       </c>
       <c r="I3" t="n">
-        <v>18260</v>
+        <v>83538</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -766,16 +762,16 @@
         </is>
       </c>
       <c r="M3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Settlement Issue</t>
+          <t>Pricing Issue</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Confirm contractual settlement date and update the incorrect record.</t>
+          <t>Review execution price, broker confirmation, and custodian booking details.</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
@@ -792,17 +788,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>T005</t>
+          <t>T0018</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Growth Fund</t>
+          <t>Short Duration Bond Fund</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>NVDA</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -812,30 +808,30 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>missing_from_custodian</t>
+          <t>settlement_date_mismatch</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Present</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Missing</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="I4" t="n">
-        <v>4910</v>
+        <v>63445.50000000001</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -844,16 +840,16 @@
         </is>
       </c>
       <c r="M4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>Booking Issue</t>
+          <t>Settlement Issue</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>Confirm record with custodian and investigate whether the position or trade failed to book externally.</t>
+          <t>Confirm contractual settlement date and update the incorrect record.</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
@@ -870,17 +866,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>T006</t>
+          <t>T0024</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Balanced Fund</t>
+          <t>Balanced Allocation Fund</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>JPM</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -890,26 +886,30 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>price_mismatch</t>
-        </is>
-      </c>
-      <c r="G5" t="n">
-        <v>205.15</v>
-      </c>
-      <c r="H5" t="n">
-        <v>204.9</v>
+          <t>currency_mismatch</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
       </c>
       <c r="I5" t="n">
-        <v>12309</v>
+        <v>10521</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -918,16 +918,16 @@
         </is>
       </c>
       <c r="M5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>Pricing Issue</t>
+          <t>Currency / FX Issue</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>Review execution price, broker confirmation, and custodian booking details.</t>
+          <t>Confirm currency and FX treatment.</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
@@ -944,50 +944,50 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>T008</t>
+          <t>T0030</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Growth Fund</t>
+          <t>Balanced Allocation Fund</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>GOOGL</t>
+          <t>XLF</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Equity</t>
+          <t>ETF</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>missing_from_custodian</t>
+          <t>side_mismatch</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Present</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Missing</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="I6" t="n">
-        <v>4455</v>
+        <v>6558</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -996,16 +996,16 @@
         </is>
       </c>
       <c r="M6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>Booking Issue</t>
+          <t>Allocation Issue</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>Confirm record with custodian and investigate whether the position or trade failed to book externally.</t>
+          <t>Review buy/sell direction against order management records.</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
@@ -1022,17 +1022,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>T010</t>
+          <t>T0035</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Income Fund</t>
+          <t>Short Duration Bond Fund</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>AGG</t>
+          <t>TLT</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -1056,7 +1056,7 @@
         </is>
       </c>
       <c r="I7" t="n">
-        <v>29280</v>
+        <v>45335</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
@@ -1100,41 +1100,41 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>T011</t>
+          <t>T0041</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Growth Fund</t>
+          <t>International Equity Fund</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>AMZN</t>
+          <t>EWJ</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Equity</t>
+          <t>ETF</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>missing_from_internal</t>
+          <t>missing_from_custodian</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
+          <t>Present</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
           <t>Missing</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>Present</t>
-        </is>
-      </c>
       <c r="I8" t="n">
-        <v>5565</v>
+        <v>10395</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
@@ -1161,7 +1161,7 @@
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>Review custodian activity and confirm whether the record should be booked internally.</t>
+          <t>Confirm record with custodian and investigate whether the position or trade failed to book externally.</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
@@ -1173,69 +1173,73 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Position Reconciliation</t>
+          <t>Trade Reconciliation</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Balanced Fund-JPM</t>
+          <t>T0048</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Balanced Fund</t>
+          <t>US Growth Fund</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>JPM</t>
+          <t>SPY</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Equity</t>
+          <t>ETF</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>market_price_mismatch</t>
-        </is>
-      </c>
-      <c r="G9" t="n">
-        <v>205.15</v>
-      </c>
-      <c r="H9" t="n">
-        <v>204.9</v>
+          <t>missing_from_custodian</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Present</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
       </c>
       <c r="I9" t="n">
-        <v>51287.5</v>
+        <v>53216.99999999999</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>Portfolio Accounting Team</t>
+          <t>Trade Operations Team</t>
         </is>
       </c>
       <c r="M9" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>Pricing Issue</t>
+          <t>Booking Issue</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>Review pricing source, valuation date, and custodian market price feed.</t>
+          <t>Confirm record with custodian and investigate whether the position or trade failed to book externally.</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
@@ -1247,17 +1251,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Position Reconciliation</t>
+          <t>Trade Reconciliation</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Growth Fund-AMZN</t>
+          <t>T0051</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Growth Fund</t>
+          <t>US Growth Fund</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1286,7 +1290,7 @@
         </is>
       </c>
       <c r="I10" t="n">
-        <v>5565</v>
+        <v>13912.5</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
@@ -1300,7 +1304,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>Portfolio Accounting Team</t>
+          <t>Trade Operations Team</t>
         </is>
       </c>
       <c r="M10" t="n">
@@ -1330,50 +1334,46 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Growth Fund-GOOGL</t>
+          <t>Balanced Allocation Fund-XLF</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Growth Fund</t>
+          <t>Balanced Allocation Fund</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>GOOGL</t>
+          <t>XLF</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Equity</t>
+          <t>ETF</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>missing_from_custodian</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>Present</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>Missing</t>
-        </is>
+          <t>market_price_mismatch</t>
+        </is>
+      </c>
+      <c r="G11" t="n">
+        <v>43.75</v>
+      </c>
+      <c r="H11" t="n">
+        <v>44.25</v>
       </c>
       <c r="I11" t="n">
-        <v>17820</v>
+        <v>8750</v>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
@@ -1382,16 +1382,16 @@
         </is>
       </c>
       <c r="M11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>Booking Issue</t>
+          <t>Pricing Issue</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>Confirm record with custodian and investigate whether the position or trade failed to book externally.</t>
+          <t>Review pricing source, valuation date, and custodian market price feed.</t>
         </is>
       </c>
       <c r="P11" t="inlineStr">
@@ -1408,17 +1408,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Growth Fund-MSFT</t>
+          <t>Core Income Fund-ASML</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Growth Fund</t>
+          <t>Core Income Fund</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>ASML</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1428,26 +1428,30 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>quantity_mismatch</t>
-        </is>
-      </c>
-      <c r="G12" t="n">
-        <v>300</v>
-      </c>
-      <c r="H12" t="n">
-        <v>295</v>
+          <t>currency_mismatch</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
       </c>
       <c r="I12" t="n">
-        <v>126030</v>
+        <v>210420</v>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
@@ -1456,16 +1460,16 @@
         </is>
       </c>
       <c r="M12" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>Allocation Issue</t>
+          <t>Currency / FX Issue</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>Compare internal allocation records against custodian position or trade details.</t>
+          <t>Confirm currency and FX treatment.</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
@@ -1482,22 +1486,22 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Income Fund-AGG</t>
+          <t>International Equity Fund-MSFT</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Income Fund</t>
+          <t>International Equity Fund</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>AGG</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Bond ETF</t>
+          <t>Equity</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1516,7 +1520,7 @@
         </is>
       </c>
       <c r="I13" t="n">
-        <v>87840</v>
+        <v>73517.5</v>
       </c>
       <c r="J13" t="inlineStr">
         <is>
@@ -1560,17 +1564,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Income Fund-IEF</t>
+          <t>Short Duration Bond Fund-TLT</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Income Fund</t>
+          <t>Short Duration Bond Fund</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>IEF</t>
+          <t>TLT</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1580,17 +1584,21 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>quantity_mismatch</t>
-        </is>
-      </c>
-      <c r="G14" t="n">
-        <v>600</v>
-      </c>
-      <c r="H14" t="n">
-        <v>610</v>
+          <t>missing_from_custodian</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Present</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
       </c>
       <c r="I14" t="n">
-        <v>56880</v>
+        <v>25107.5</v>
       </c>
       <c r="J14" t="inlineStr">
         <is>
@@ -1599,7 +1607,7 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>High</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
@@ -1608,16 +1616,16 @@
         </is>
       </c>
       <c r="M14" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>Allocation Issue</t>
+          <t>Booking Issue</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>Compare internal allocation records against custodian position or trade details.</t>
+          <t>Confirm record with custodian and investigate whether the position or trade failed to book externally.</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
@@ -1629,42 +1637,46 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Cash Reconciliation</t>
+          <t>Position Reconciliation</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Growth Fund-USD</t>
+          <t>US Growth Fund-AMZN</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Growth Fund</t>
+          <t>US Growth Fund</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Cash</t>
+          <t>AMZN</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Cash</t>
+          <t>Equity</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>cash_balance_mismatch</t>
-        </is>
-      </c>
-      <c r="G15" t="n">
-        <v>125000</v>
-      </c>
-      <c r="H15" t="n">
-        <v>119435</v>
+          <t>missing_from_internal</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Present</t>
+        </is>
       </c>
       <c r="I15" t="n">
-        <v>5565</v>
+        <v>18550</v>
       </c>
       <c r="J15" t="inlineStr">
         <is>
@@ -1678,7 +1690,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>Cash Operations Team</t>
+          <t>Portfolio Accounting Team</t>
         </is>
       </c>
       <c r="M15" t="n">
@@ -1686,12 +1698,12 @@
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>Cash Movement Issue</t>
+          <t>Booking Issue</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>Investigate unsettled trades, custodian cash movements, fees, and income activity causing the cash difference.</t>
+          <t>Review custodian activity and confirm whether the record should be booked internally.</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
@@ -1703,42 +1715,42 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Cash Reconciliation</t>
+          <t>Position Reconciliation</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Income Fund-USD</t>
+          <t>US Growth Fund-NVDA</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Income Fund</t>
+          <t>US Growth Fund</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Cash</t>
+          <t>NVDA</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Cash</t>
+          <t>Equity</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>cash_balance_mismatch</t>
+          <t>quantity_mismatch</t>
         </is>
       </c>
       <c r="G16" t="n">
-        <v>152500</v>
+        <v>250</v>
       </c>
       <c r="H16" t="n">
-        <v>123220</v>
+        <v>225</v>
       </c>
       <c r="I16" t="n">
-        <v>29280</v>
+        <v>30687.5</v>
       </c>
       <c r="J16" t="inlineStr">
         <is>
@@ -1752,7 +1764,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>Cash Operations Team</t>
+          <t>Portfolio Accounting Team</t>
         </is>
       </c>
       <c r="M16" t="n">
@@ -1760,15 +1772,163 @@
       </c>
       <c r="N16" t="inlineStr">
         <is>
+          <t>Allocation Issue</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>Compare internal allocation records against custodian position or trade details.</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Cash Reconciliation</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Growth Fund-USD</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Growth Fund</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>cash_balance_mismatch</t>
+        </is>
+      </c>
+      <c r="G17" t="n">
+        <v>125000</v>
+      </c>
+      <c r="H17" t="n">
+        <v>119435</v>
+      </c>
+      <c r="I17" t="n">
+        <v>5565</v>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>Cash Operations Team</t>
+        </is>
+      </c>
+      <c r="M17" t="n">
+        <v>2</v>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
           <t>Cash Movement Issue</t>
         </is>
       </c>
-      <c r="O16" t="inlineStr">
+      <c r="O17" t="inlineStr">
         <is>
           <t>Investigate unsettled trades, custodian cash movements, fees, and income activity causing the cash difference.</t>
         </is>
       </c>
-      <c r="P16" t="inlineStr">
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Cash Reconciliation</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Income Fund-USD</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Income Fund</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>cash_balance_mismatch</t>
+        </is>
+      </c>
+      <c r="G18" t="n">
+        <v>152500</v>
+      </c>
+      <c r="H18" t="n">
+        <v>123220</v>
+      </c>
+      <c r="I18" t="n">
+        <v>29280</v>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>Cash Operations Team</t>
+        </is>
+      </c>
+      <c r="M18" t="n">
+        <v>2</v>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>Cash Movement Issue</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>Investigate unsettled trades, custodian cash movements, fees, and income activity causing the cash difference.</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -1785,7 +1945,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P8"/>
+  <dimension ref="A1:P10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1878,17 +2038,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>T002</t>
+          <t>T0007</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Growth Fund</t>
+          <t>Short Duration Bond Fund</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>JPM</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -1902,13 +2062,13 @@
         </is>
       </c>
       <c r="G2" t="n">
-        <v>75</v>
+        <v>200</v>
       </c>
       <c r="H2" t="n">
-        <v>70</v>
+        <v>175</v>
       </c>
       <c r="I2" t="n">
-        <v>31507.5</v>
+        <v>41094</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -1952,50 +2112,46 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>T004</t>
+          <t>T0012</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Income Fund</t>
+          <t>Core Income Fund</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>TLT</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Bond ETF</t>
+          <t>Equity</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>settlement_date_mismatch</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>2026-06-04</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>2026-06-05</t>
-        </is>
+          <t>price_mismatch</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>417.69</v>
+      </c>
+      <c r="H3" t="n">
+        <v>418.04</v>
       </c>
       <c r="I3" t="n">
-        <v>18260</v>
+        <v>83538</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -2004,16 +2160,16 @@
         </is>
       </c>
       <c r="M3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Settlement Issue</t>
+          <t>Pricing Issue</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Confirm contractual settlement date and update the incorrect record.</t>
+          <t>Review execution price, broker confirmation, and custodian booking details.</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
@@ -2030,17 +2186,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>T005</t>
+          <t>T0018</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Growth Fund</t>
+          <t>Short Duration Bond Fund</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>NVDA</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -2050,30 +2206,30 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>missing_from_custodian</t>
+          <t>settlement_date_mismatch</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Present</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Missing</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="I4" t="n">
-        <v>4910</v>
+        <v>63445.50000000001</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -2082,16 +2238,16 @@
         </is>
       </c>
       <c r="M4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>Booking Issue</t>
+          <t>Settlement Issue</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>Confirm record with custodian and investigate whether the position or trade failed to book externally.</t>
+          <t>Confirm contractual settlement date and update the incorrect record.</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
@@ -2108,17 +2264,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>T006</t>
+          <t>T0024</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Balanced Fund</t>
+          <t>Balanced Allocation Fund</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>JPM</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -2128,26 +2284,30 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>price_mismatch</t>
-        </is>
-      </c>
-      <c r="G5" t="n">
-        <v>205.15</v>
-      </c>
-      <c r="H5" t="n">
-        <v>204.9</v>
+          <t>currency_mismatch</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
       </c>
       <c r="I5" t="n">
-        <v>12309</v>
+        <v>10521</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -2156,16 +2316,16 @@
         </is>
       </c>
       <c r="M5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>Pricing Issue</t>
+          <t>Currency / FX Issue</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>Review execution price, broker confirmation, and custodian booking details.</t>
+          <t>Confirm currency and FX treatment.</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
@@ -2182,50 +2342,50 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>T008</t>
+          <t>T0030</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Growth Fund</t>
+          <t>Balanced Allocation Fund</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>GOOGL</t>
+          <t>XLF</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Equity</t>
+          <t>ETF</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>missing_from_custodian</t>
+          <t>side_mismatch</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Present</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Missing</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="I6" t="n">
-        <v>4455</v>
+        <v>6558</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -2234,16 +2394,16 @@
         </is>
       </c>
       <c r="M6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>Booking Issue</t>
+          <t>Allocation Issue</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>Confirm record with custodian and investigate whether the position or trade failed to book externally.</t>
+          <t>Review buy/sell direction against order management records.</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
@@ -2260,17 +2420,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>T010</t>
+          <t>T0035</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Income Fund</t>
+          <t>Short Duration Bond Fund</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>AGG</t>
+          <t>TLT</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -2294,7 +2454,7 @@
         </is>
       </c>
       <c r="I7" t="n">
-        <v>29280</v>
+        <v>45335</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
@@ -2338,41 +2498,41 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>T011</t>
+          <t>T0041</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Growth Fund</t>
+          <t>International Equity Fund</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>AMZN</t>
+          <t>EWJ</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Equity</t>
+          <t>ETF</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>missing_from_internal</t>
+          <t>missing_from_custodian</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
+          <t>Present</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
           <t>Missing</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>Present</t>
-        </is>
-      </c>
       <c r="I8" t="n">
-        <v>5565</v>
+        <v>10395</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
@@ -2399,10 +2559,166 @@
       </c>
       <c r="O8" t="inlineStr">
         <is>
+          <t>Confirm record with custodian and investigate whether the position or trade failed to book externally.</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Trade Reconciliation</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>T0048</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>US Growth Fund</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>ETF</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>missing_from_custodian</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Present</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>53216.99999999999</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>Trade Operations Team</t>
+        </is>
+      </c>
+      <c r="M9" t="n">
+        <v>4</v>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>Booking Issue</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>Confirm record with custodian and investigate whether the position or trade failed to book externally.</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Trade Reconciliation</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>T0051</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>US Growth Fund</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Equity</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>missing_from_internal</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Present</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>13912.5</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>Trade Operations Team</t>
+        </is>
+      </c>
+      <c r="M10" t="n">
+        <v>2</v>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>Booking Issue</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
           <t>Review custodian activity and confirm whether the record should be booked internally.</t>
         </is>
       </c>
-      <c r="P8" t="inlineStr">
+      <c r="P10" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -2512,22 +2828,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Balanced Fund-JPM</t>
+          <t>Balanced Allocation Fund-XLF</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Balanced Fund</t>
+          <t>Balanced Allocation Fund</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>JPM</t>
+          <t>XLF</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Equity</t>
+          <t>ETF</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -2536,13 +2852,13 @@
         </is>
       </c>
       <c r="G2" t="n">
-        <v>205.15</v>
+        <v>43.75</v>
       </c>
       <c r="H2" t="n">
-        <v>204.9</v>
+        <v>44.25</v>
       </c>
       <c r="I2" t="n">
-        <v>51287.5</v>
+        <v>8750</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -2586,17 +2902,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Growth Fund-AMZN</t>
+          <t>Core Income Fund-ASML</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Growth Fund</t>
+          <t>Core Income Fund</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>AMZN</t>
+          <t>ASML</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -2606,30 +2922,30 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>missing_from_internal</t>
+          <t>currency_mismatch</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Missing</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Present</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="I3" t="n">
-        <v>5565</v>
+        <v>210420</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -2638,16 +2954,16 @@
         </is>
       </c>
       <c r="M3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Booking Issue</t>
+          <t>Currency / FX Issue</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Review custodian activity and confirm whether the record should be booked internally.</t>
+          <t>Confirm currency and FX treatment.</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
@@ -2664,17 +2980,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Growth Fund-GOOGL</t>
+          <t>International Equity Fund-MSFT</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Growth Fund</t>
+          <t>International Equity Fund</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>GOOGL</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -2698,7 +3014,7 @@
         </is>
       </c>
       <c r="I4" t="n">
-        <v>17820</v>
+        <v>73517.5</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
@@ -2707,7 +3023,7 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -2716,7 +3032,7 @@
         </is>
       </c>
       <c r="M4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N4" t="inlineStr">
         <is>
@@ -2742,37 +3058,41 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Growth Fund-MSFT</t>
+          <t>Short Duration Bond Fund-TLT</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Growth Fund</t>
+          <t>Short Duration Bond Fund</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>TLT</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Equity</t>
+          <t>Bond ETF</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>quantity_mismatch</t>
-        </is>
-      </c>
-      <c r="G5" t="n">
-        <v>300</v>
-      </c>
-      <c r="H5" t="n">
-        <v>295</v>
+          <t>missing_from_custodian</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Present</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
       </c>
       <c r="I5" t="n">
-        <v>126030</v>
+        <v>25107.5</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
@@ -2781,7 +3101,7 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>High</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -2790,16 +3110,16 @@
         </is>
       </c>
       <c r="M5" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>Allocation Issue</t>
+          <t>Booking Issue</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>Compare internal allocation records against custodian position or trade details.</t>
+          <t>Confirm record with custodian and investigate whether the position or trade failed to book externally.</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
@@ -2816,41 +3136,41 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Income Fund-AGG</t>
+          <t>US Growth Fund-AMZN</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Income Fund</t>
+          <t>US Growth Fund</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>AGG</t>
+          <t>AMZN</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Bond ETF</t>
+          <t>Equity</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>missing_from_custodian</t>
+          <t>missing_from_internal</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
           <t>Present</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>Missing</t>
-        </is>
-      </c>
       <c r="I6" t="n">
-        <v>87840</v>
+        <v>18550</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
@@ -2859,7 +3179,7 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>High</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -2868,7 +3188,7 @@
         </is>
       </c>
       <c r="M6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N6" t="inlineStr">
         <is>
@@ -2877,7 +3197,7 @@
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>Confirm record with custodian and investigate whether the position or trade failed to book externally.</t>
+          <t>Review custodian activity and confirm whether the record should be booked internally.</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
@@ -2894,22 +3214,22 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Income Fund-IEF</t>
+          <t>US Growth Fund-NVDA</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Income Fund</t>
+          <t>US Growth Fund</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>IEF</t>
+          <t>NVDA</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Bond ETF</t>
+          <t>Equity</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -2918,13 +3238,13 @@
         </is>
       </c>
       <c r="G7" t="n">
-        <v>600</v>
+        <v>250</v>
       </c>
       <c r="H7" t="n">
-        <v>610</v>
+        <v>225</v>
       </c>
       <c r="I7" t="n">
-        <v>56880</v>
+        <v>30687.5</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
@@ -2933,7 +3253,7 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>High</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -2942,7 +3262,7 @@
         </is>
       </c>
       <c r="M7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N7" t="inlineStr">
         <is>
@@ -3215,7 +3535,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P14"/>
+  <dimension ref="A1:P13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3303,17 +3623,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Position Reconciliation</t>
+          <t>Trade Reconciliation</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Growth Fund-MSFT</t>
+          <t>T0012</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Growth Fund</t>
+          <t>Core Income Fund</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -3328,17 +3648,17 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>quantity_mismatch</t>
+          <t>price_mismatch</t>
         </is>
       </c>
       <c r="G2" t="n">
-        <v>300</v>
+        <v>417.69</v>
       </c>
       <c r="H2" t="n">
-        <v>295</v>
+        <v>418.04</v>
       </c>
       <c r="I2" t="n">
-        <v>126030</v>
+        <v>83538</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -3352,7 +3672,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Portfolio Accounting Team</t>
+          <t>Trade Operations Team</t>
         </is>
       </c>
       <c r="M2" t="n">
@@ -3360,12 +3680,12 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>Allocation Issue</t>
+          <t>Pricing Issue</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>Compare internal allocation records against custodian position or trade details.</t>
+          <t>Review execution price, broker confirmation, and custodian booking details.</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
@@ -3382,22 +3702,22 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Income Fund-AGG</t>
+          <t>International Equity Fund-MSFT</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Income Fund</t>
+          <t>International Equity Fund</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>AGG</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Bond ETF</t>
+          <t>Equity</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -3416,7 +3736,7 @@
         </is>
       </c>
       <c r="I3" t="n">
-        <v>87840</v>
+        <v>73517.5</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
@@ -3455,42 +3775,46 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Position Reconciliation</t>
+          <t>Trade Reconciliation</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Income Fund-IEF</t>
+          <t>T0048</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Income Fund</t>
+          <t>US Growth Fund</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>IEF</t>
+          <t>SPY</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Bond ETF</t>
+          <t>ETF</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>quantity_mismatch</t>
-        </is>
-      </c>
-      <c r="G4" t="n">
-        <v>600</v>
-      </c>
-      <c r="H4" t="n">
-        <v>610</v>
+          <t>missing_from_custodian</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Present</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
       </c>
       <c r="I4" t="n">
-        <v>56880</v>
+        <v>53216.99999999999</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
@@ -3504,7 +3828,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>Portfolio Accounting Team</t>
+          <t>Trade Operations Team</t>
         </is>
       </c>
       <c r="M4" t="n">
@@ -3512,12 +3836,12 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>Allocation Issue</t>
+          <t>Booking Issue</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>Compare internal allocation records against custodian position or trade details.</t>
+          <t>Confirm record with custodian and investigate whether the position or trade failed to book externally.</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
@@ -3534,37 +3858,41 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>T002</t>
+          <t>T0035</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Growth Fund</t>
+          <t>Short Duration Bond Fund</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>TLT</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Equity</t>
+          <t>Bond ETF</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>quantity_mismatch</t>
-        </is>
-      </c>
-      <c r="G5" t="n">
-        <v>75</v>
-      </c>
-      <c r="H5" t="n">
-        <v>70</v>
+          <t>missing_from_custodian</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Present</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
       </c>
       <c r="I5" t="n">
-        <v>31507.5</v>
+        <v>45335</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
@@ -3586,12 +3914,12 @@
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>Allocation Issue</t>
+          <t>Booking Issue</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>Compare internal allocation records against custodian position or trade details.</t>
+          <t>Confirm record with custodian and investigate whether the position or trade failed to book externally.</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
@@ -3608,41 +3936,37 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>T010</t>
+          <t>T0007</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Income Fund</t>
+          <t>Short Duration Bond Fund</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>AGG</t>
+          <t>JPM</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Bond ETF</t>
+          <t>Equity</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>missing_from_custodian</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>Present</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>Missing</t>
-        </is>
+          <t>quantity_mismatch</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>200</v>
+      </c>
+      <c r="H6" t="n">
+        <v>175</v>
       </c>
       <c r="I6" t="n">
-        <v>29280</v>
+        <v>41094</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
@@ -3664,12 +3988,12 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>Booking Issue</t>
+          <t>Allocation Issue</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>Confirm record with custodian and investigate whether the position or trade failed to book externally.</t>
+          <t>Compare internal allocation records against custodian position or trade details.</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
@@ -3681,42 +4005,42 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Cash Reconciliation</t>
+          <t>Position Reconciliation</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Income Fund-USD</t>
+          <t>US Growth Fund-NVDA</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Income Fund</t>
+          <t>US Growth Fund</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Cash</t>
+          <t>NVDA</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Cash</t>
+          <t>Equity</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>cash_balance_mismatch</t>
+          <t>quantity_mismatch</t>
         </is>
       </c>
       <c r="G7" t="n">
-        <v>152500</v>
+        <v>250</v>
       </c>
       <c r="H7" t="n">
-        <v>123220</v>
+        <v>225</v>
       </c>
       <c r="I7" t="n">
-        <v>29280</v>
+        <v>30687.5</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
@@ -3730,7 +4054,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>Cash Operations Team</t>
+          <t>Portfolio Accounting Team</t>
         </is>
       </c>
       <c r="M7" t="n">
@@ -3738,12 +4062,12 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>Cash Movement Issue</t>
+          <t>Allocation Issue</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>Investigate unsettled trades, custodian cash movements, fees, and income activity causing the cash difference.</t>
+          <t>Compare internal allocation records against custodian position or trade details.</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
@@ -3755,46 +4079,42 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Position Reconciliation</t>
+          <t>Cash Reconciliation</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Growth Fund-GOOGL</t>
+          <t>Income Fund-USD</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Growth Fund</t>
+          <t>Income Fund</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>GOOGL</t>
+          <t>Cash</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Equity</t>
+          <t>Cash</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>missing_from_custodian</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>Present</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>Missing</t>
-        </is>
+          <t>cash_balance_mismatch</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
+        <v>152500</v>
+      </c>
+      <c r="H8" t="n">
+        <v>123220</v>
       </c>
       <c r="I8" t="n">
-        <v>17820</v>
+        <v>29280</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
@@ -3808,7 +4128,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>Portfolio Accounting Team</t>
+          <t>Cash Operations Team</t>
         </is>
       </c>
       <c r="M8" t="n">
@@ -3816,12 +4136,12 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>Booking Issue</t>
+          <t>Cash Movement Issue</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>Confirm record with custodian and investigate whether the position or trade failed to book externally.</t>
+          <t>Investigate unsettled trades, custodian cash movements, fees, and income activity causing the cash difference.</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
@@ -3833,42 +4153,46 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Trade Reconciliation</t>
+          <t>Position Reconciliation</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>T006</t>
+          <t>Short Duration Bond Fund-TLT</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Balanced Fund</t>
+          <t>Short Duration Bond Fund</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>JPM</t>
+          <t>TLT</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Equity</t>
+          <t>Bond ETF</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>price_mismatch</t>
-        </is>
-      </c>
-      <c r="G9" t="n">
-        <v>205.15</v>
-      </c>
-      <c r="H9" t="n">
-        <v>204.9</v>
+          <t>missing_from_custodian</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Present</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
       </c>
       <c r="I9" t="n">
-        <v>12309</v>
+        <v>25107.5</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
@@ -3882,7 +4206,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>Trade Operations Team</t>
+          <t>Portfolio Accounting Team</t>
         </is>
       </c>
       <c r="M9" t="n">
@@ -3890,12 +4214,12 @@
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>Pricing Issue</t>
+          <t>Booking Issue</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>Review execution price, broker confirmation, and custodian booking details.</t>
+          <t>Confirm record with custodian and investigate whether the position or trade failed to book externally.</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
@@ -3912,12 +4236,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Growth Fund-AMZN</t>
+          <t>US Growth Fund-AMZN</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Growth Fund</t>
+          <t>US Growth Fund</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -3946,7 +4270,7 @@
         </is>
       </c>
       <c r="I10" t="n">
-        <v>5565</v>
+        <v>18550</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
@@ -3990,12 +4314,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>T011</t>
+          <t>T0051</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Growth Fund</t>
+          <t>US Growth Fund</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -4024,7 +4348,7 @@
         </is>
       </c>
       <c r="I11" t="n">
-        <v>5565</v>
+        <v>13912.5</v>
       </c>
       <c r="J11" t="inlineStr">
         <is>
@@ -4063,42 +4387,46 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Cash Reconciliation</t>
+          <t>Trade Reconciliation</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Growth Fund-USD</t>
+          <t>T0041</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Growth Fund</t>
+          <t>International Equity Fund</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Cash</t>
+          <t>EWJ</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Cash</t>
+          <t>ETF</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>cash_balance_mismatch</t>
-        </is>
-      </c>
-      <c r="G12" t="n">
-        <v>125000</v>
-      </c>
-      <c r="H12" t="n">
-        <v>119435</v>
+          <t>missing_from_custodian</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Present</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
       </c>
       <c r="I12" t="n">
-        <v>5565</v>
+        <v>10395</v>
       </c>
       <c r="J12" t="inlineStr">
         <is>
@@ -4112,7 +4440,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>Cash Operations Team</t>
+          <t>Trade Operations Team</t>
         </is>
       </c>
       <c r="M12" t="n">
@@ -4120,12 +4448,12 @@
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>Cash Movement Issue</t>
+          <t>Booking Issue</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>Investigate unsettled trades, custodian cash movements, fees, and income activity causing the cash difference.</t>
+          <t>Confirm record with custodian and investigate whether the position or trade failed to book externally.</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
@@ -4137,12 +4465,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Trade Reconciliation</t>
+          <t>Cash Reconciliation</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>T005</t>
+          <t>Growth Fund-USD</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -4152,31 +4480,27 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>NVDA</t>
+          <t>Cash</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Equity</t>
+          <t>Cash</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>missing_from_custodian</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>Present</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>Missing</t>
-        </is>
+          <t>cash_balance_mismatch</t>
+        </is>
+      </c>
+      <c r="G13" t="n">
+        <v>125000</v>
+      </c>
+      <c r="H13" t="n">
+        <v>119435</v>
       </c>
       <c r="I13" t="n">
-        <v>4910</v>
+        <v>5565</v>
       </c>
       <c r="J13" t="inlineStr">
         <is>
@@ -4190,7 +4514,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>Trade Operations Team</t>
+          <t>Cash Operations Team</t>
         </is>
       </c>
       <c r="M13" t="n">
@@ -4198,93 +4522,15 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>Booking Issue</t>
+          <t>Cash Movement Issue</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>Confirm record with custodian and investigate whether the position or trade failed to book externally.</t>
+          <t>Investigate unsettled trades, custodian cash movements, fees, and income activity causing the cash difference.</t>
         </is>
       </c>
       <c r="P13" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Trade Reconciliation</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>T008</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Growth Fund</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>GOOGL</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>Equity</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>missing_from_custodian</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>Present</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="I14" t="n">
-        <v>4455</v>
-      </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="L14" t="inlineStr">
-        <is>
-          <t>Trade Operations Team</t>
-        </is>
-      </c>
-      <c r="M14" t="n">
-        <v>2</v>
-      </c>
-      <c r="N14" t="inlineStr">
-        <is>
-          <t>Booking Issue</t>
-        </is>
-      </c>
-      <c r="O14" t="inlineStr">
-        <is>
-          <t>Confirm record with custodian and investigate whether the position or trade failed to book externally.</t>
-        </is>
-      </c>
-      <c r="P14" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -4301,7 +4547,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4329,49 +4575,113 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Income Fund</t>
+          <t>Core Income Fund</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D2" t="n">
-        <v>221540</v>
+        <v>293958</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Growth Fund</t>
+          <t>Short Duration Bond Fund</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="C3" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="D3" t="n">
-        <v>201417.5</v>
+        <v>174982</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Balanced Fund</t>
+          <t>US Growth Fund</t>
         </is>
       </c>
       <c r="B4" t="n">
+        <v>4</v>
+      </c>
+      <c r="C4" t="n">
+        <v>4</v>
+      </c>
+      <c r="D4" t="n">
+        <v>116367</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>International Equity Fund</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
         <v>2</v>
       </c>
-      <c r="C4" t="n">
+      <c r="C5" t="n">
+        <v>2</v>
+      </c>
+      <c r="D5" t="n">
+        <v>83912.5</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Income Fund</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
         <v>1</v>
       </c>
-      <c r="D4" t="n">
-        <v>63596.5</v>
+      <c r="C6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" t="n">
+        <v>29280</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Balanced Allocation Fund</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>3</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" t="n">
+        <v>25829</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Growth Fund</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>1</v>
+      </c>
+      <c r="C8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" t="n">
+        <v>5565</v>
       </c>
     </row>
   </sheetData>
@@ -4415,7 +4725,7 @@
         <v>6</v>
       </c>
       <c r="C2" t="n">
-        <v>345422.5</v>
+        <v>367032.5</v>
       </c>
     </row>
     <row r="3">
@@ -4425,10 +4735,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C3" t="n">
-        <v>106286.5</v>
+        <v>328016</v>
       </c>
     </row>
     <row r="4">
@@ -4455,7 +4765,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4478,27 +4788,27 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Allocation Issue</t>
+          <t>Booking Issue</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="C2" t="n">
-        <v>214417.5</v>
+        <v>240034.5</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Booking Issue</t>
+          <t>Currency / FX Issue</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="C3" t="n">
-        <v>155435</v>
+        <v>220941</v>
       </c>
     </row>
     <row r="4">
@@ -4511,20 +4821,20 @@
         <v>2</v>
       </c>
       <c r="C4" t="n">
-        <v>63596.5</v>
+        <v>92288</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Cash Movement Issue</t>
+          <t>Allocation Issue</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C5" t="n">
-        <v>34845</v>
+        <v>78339.5</v>
       </c>
     </row>
     <row r="6">
@@ -4537,7 +4847,20 @@
         <v>1</v>
       </c>
       <c r="C6" t="n">
-        <v>18260</v>
+        <v>63445.50000000001</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Cash Movement Issue</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>2</v>
+      </c>
+      <c r="C7" t="n">
+        <v>34845</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Generate and connect expanded cash dataset
</commit_message>
<xml_diff>
--- a/output/Investment_Operations_Exception_Report.xlsx
+++ b/output/Investment_Operations_Exception_Report.xlsx
@@ -443,7 +443,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="3">
@@ -473,7 +473,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6">
@@ -493,7 +493,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="8">
@@ -513,7 +513,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>729893.5</v>
+        <v>742998.5</v>
       </c>
     </row>
     <row r="10">
@@ -533,7 +533,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>2.6</v>
+        <v>2.7</v>
       </c>
     </row>
   </sheetData>
@@ -547,7 +547,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P18"/>
+  <dimension ref="A1:P19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1794,12 +1794,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Growth Fund-USD</t>
+          <t>Core Income Fund-USD</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Growth Fund</t>
+          <t>Core Income Fund</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1818,13 +1818,13 @@
         </is>
       </c>
       <c r="G17" t="n">
-        <v>125000</v>
+        <v>410000</v>
       </c>
       <c r="H17" t="n">
-        <v>119435</v>
+        <v>439400</v>
       </c>
       <c r="I17" t="n">
-        <v>5565</v>
+        <v>29400</v>
       </c>
       <c r="J17" t="inlineStr">
         <is>
@@ -1868,12 +1868,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Income Fund-USD</t>
+          <t>International Equity Fund-USD</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Income Fund</t>
+          <t>International Equity Fund</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1888,47 +1888,125 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
+          <t>as_of_date_mismatch</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
+        <v>0</v>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>Cash Operations Team</t>
+        </is>
+      </c>
+      <c r="M18" t="n">
+        <v>3</v>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>Data Quality Issue</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>Confirm both cash balances are using the same valuation date.</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Cash Reconciliation</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>US Growth Fund-USD</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>US Growth Fund</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
           <t>cash_balance_mismatch</t>
         </is>
       </c>
-      <c r="G18" t="n">
-        <v>152500</v>
-      </c>
-      <c r="H18" t="n">
-        <v>123220</v>
-      </c>
-      <c r="I18" t="n">
-        <v>29280</v>
-      </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="L18" t="inlineStr">
+      <c r="G19" t="n">
+        <v>250000</v>
+      </c>
+      <c r="H19" t="n">
+        <v>231450</v>
+      </c>
+      <c r="I19" t="n">
+        <v>18550</v>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
         <is>
           <t>Cash Operations Team</t>
         </is>
       </c>
-      <c r="M18" t="n">
+      <c r="M19" t="n">
         <v>2</v>
       </c>
-      <c r="N18" t="inlineStr">
+      <c r="N19" t="inlineStr">
         <is>
           <t>Cash Movement Issue</t>
         </is>
       </c>
-      <c r="O18" t="inlineStr">
+      <c r="O19" t="inlineStr">
         <is>
           <t>Investigate unsettled trades, custodian cash movements, fees, and income activity causing the cash difference.</t>
         </is>
       </c>
-      <c r="P18" t="inlineStr">
+      <c r="P19" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -3291,7 +3369,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P3"/>
+  <dimension ref="A1:P4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3384,12 +3462,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Growth Fund-USD</t>
+          <t>Core Income Fund-USD</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Growth Fund</t>
+          <t>Core Income Fund</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -3408,13 +3486,13 @@
         </is>
       </c>
       <c r="G2" t="n">
-        <v>125000</v>
+        <v>410000</v>
       </c>
       <c r="H2" t="n">
-        <v>119435</v>
+        <v>439400</v>
       </c>
       <c r="I2" t="n">
-        <v>5565</v>
+        <v>29400</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -3458,12 +3536,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Income Fund-USD</t>
+          <t>International Equity Fund-USD</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Income Fund</t>
+          <t>International Equity Fund</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -3478,47 +3556,125 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
+          <t>as_of_date_mismatch</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="I3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Cash Operations Team</t>
+        </is>
+      </c>
+      <c r="M3" t="n">
+        <v>3</v>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Data Quality Issue</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>Confirm both cash balances are using the same valuation date.</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Cash Reconciliation</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>US Growth Fund-USD</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>US Growth Fund</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
           <t>cash_balance_mismatch</t>
         </is>
       </c>
-      <c r="G3" t="n">
-        <v>152500</v>
-      </c>
-      <c r="H3" t="n">
-        <v>123220</v>
-      </c>
-      <c r="I3" t="n">
-        <v>29280</v>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
+      <c r="G4" t="n">
+        <v>250000</v>
+      </c>
+      <c r="H4" t="n">
+        <v>231450</v>
+      </c>
+      <c r="I4" t="n">
+        <v>18550</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
         <is>
           <t>Cash Operations Team</t>
         </is>
       </c>
-      <c r="M3" t="n">
+      <c r="M4" t="n">
         <v>2</v>
       </c>
-      <c r="N3" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t>Cash Movement Issue</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr">
+      <c r="O4" t="inlineStr">
         <is>
           <t>Investigate unsettled trades, custodian cash movements, fees, and income activity causing the cash difference.</t>
         </is>
       </c>
-      <c r="P3" t="inlineStr">
+      <c r="P4" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -4084,12 +4240,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Income Fund-USD</t>
+          <t>Core Income Fund-USD</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Income Fund</t>
+          <t>Core Income Fund</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -4108,13 +4264,13 @@
         </is>
       </c>
       <c r="G8" t="n">
-        <v>152500</v>
+        <v>410000</v>
       </c>
       <c r="H8" t="n">
-        <v>123220</v>
+        <v>439400</v>
       </c>
       <c r="I8" t="n">
-        <v>29280</v>
+        <v>29400</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
@@ -4231,12 +4387,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Position Reconciliation</t>
+          <t>Cash Reconciliation</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>US Growth Fund-AMZN</t>
+          <t>US Growth Fund-USD</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -4246,28 +4402,24 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>AMZN</t>
+          <t>Cash</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Equity</t>
+          <t>Cash</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>missing_from_internal</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>Present</t>
-        </is>
+          <t>cash_balance_mismatch</t>
+        </is>
+      </c>
+      <c r="G10" t="n">
+        <v>250000</v>
+      </c>
+      <c r="H10" t="n">
+        <v>231450</v>
       </c>
       <c r="I10" t="n">
         <v>18550</v>
@@ -4284,7 +4436,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>Portfolio Accounting Team</t>
+          <t>Cash Operations Team</t>
         </is>
       </c>
       <c r="M10" t="n">
@@ -4292,12 +4444,12 @@
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>Booking Issue</t>
+          <t>Cash Movement Issue</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>Review custodian activity and confirm whether the record should be booked internally.</t>
+          <t>Investigate unsettled trades, custodian cash movements, fees, and income activity causing the cash difference.</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
@@ -4309,12 +4461,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Trade Reconciliation</t>
+          <t>Position Reconciliation</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>T0051</t>
+          <t>US Growth Fund-AMZN</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -4348,7 +4500,7 @@
         </is>
       </c>
       <c r="I11" t="n">
-        <v>13912.5</v>
+        <v>18550</v>
       </c>
       <c r="J11" t="inlineStr">
         <is>
@@ -4362,7 +4514,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>Trade Operations Team</t>
+          <t>Portfolio Accounting Team</t>
         </is>
       </c>
       <c r="M11" t="n">
@@ -4392,41 +4544,41 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>T0041</t>
+          <t>T0051</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>International Equity Fund</t>
+          <t>US Growth Fund</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>EWJ</t>
+          <t>AMZN</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>ETF</t>
+          <t>Equity</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>missing_from_custodian</t>
+          <t>missing_from_internal</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
           <t>Present</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>Missing</t>
-        </is>
-      </c>
       <c r="I12" t="n">
-        <v>10395</v>
+        <v>13912.5</v>
       </c>
       <c r="J12" t="inlineStr">
         <is>
@@ -4453,7 +4605,7 @@
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>Confirm record with custodian and investigate whether the position or trade failed to book externally.</t>
+          <t>Review custodian activity and confirm whether the record should be booked internally.</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
@@ -4465,42 +4617,46 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Cash Reconciliation</t>
+          <t>Trade Reconciliation</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Growth Fund-USD</t>
+          <t>T0041</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Growth Fund</t>
+          <t>International Equity Fund</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Cash</t>
+          <t>EWJ</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Cash</t>
+          <t>ETF</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>cash_balance_mismatch</t>
-        </is>
-      </c>
-      <c r="G13" t="n">
-        <v>125000</v>
-      </c>
-      <c r="H13" t="n">
-        <v>119435</v>
+          <t>missing_from_custodian</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Present</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
       </c>
       <c r="I13" t="n">
-        <v>5565</v>
+        <v>10395</v>
       </c>
       <c r="J13" t="inlineStr">
         <is>
@@ -4514,7 +4670,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>Cash Operations Team</t>
+          <t>Trade Operations Team</t>
         </is>
       </c>
       <c r="M13" t="n">
@@ -4522,12 +4678,12 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>Cash Movement Issue</t>
+          <t>Booking Issue</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>Investigate unsettled trades, custodian cash movements, fees, and income activity causing the cash difference.</t>
+          <t>Confirm record with custodian and investigate whether the position or trade failed to book externally.</t>
         </is>
       </c>
       <c r="P13" t="inlineStr">
@@ -4547,7 +4703,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4579,13 +4735,13 @@
         </is>
       </c>
       <c r="B2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C2" t="n">
         <v>2</v>
       </c>
-      <c r="C2" t="n">
-        <v>1</v>
-      </c>
       <c r="D2" t="n">
-        <v>293958</v>
+        <v>323358</v>
       </c>
     </row>
     <row r="3">
@@ -4611,13 +4767,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D4" t="n">
-        <v>116367</v>
+        <v>134917</v>
       </c>
     </row>
     <row r="5">
@@ -4627,7 +4783,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C5" t="n">
         <v>2</v>
@@ -4639,49 +4795,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Income Fund</t>
+          <t>Balanced Allocation Fund</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D6" t="n">
-        <v>29280</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Balanced Allocation Fund</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>3</v>
-      </c>
-      <c r="C7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D7" t="n">
         <v>25829</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Growth Fund</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>1</v>
-      </c>
-      <c r="C8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D8" t="n">
-        <v>5565</v>
       </c>
     </row>
   </sheetData>
@@ -4748,10 +4872,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C4" t="n">
-        <v>34845</v>
+        <v>47950</v>
       </c>
     </row>
   </sheetData>
@@ -4765,7 +4889,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4860,7 +4984,20 @@
         <v>2</v>
       </c>
       <c r="C7" t="n">
-        <v>34845</v>
+        <v>47950</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Data Quality Issue</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>1</v>
+      </c>
+      <c r="C8" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>